<commit_message>
Added fourth lab and updated third lab
</commit_message>
<xml_diff>
--- a/lab3/Антонов_Артём_Сергеевич_Лаб_3.xlsx
+++ b/lab3/Антонов_Артём_Сергеевич_Лаб_3.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Canon\Desktop\лабы_информ\Лаба3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\student\Downloads\lab_informatics-master\lab_informatics-master\lab3\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11250" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12555" windowHeight="3195" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Лист6" sheetId="6" r:id="rId6"/>
     <sheet name="Лист7" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="70">
   <si>
     <t>ВЫЧИСЛЕНИЯ ПО ФОРМУЛАМ С ИСПОЛЬЗОВАНИЕМ ВСТРОЕННЫХ МАТЕМАТИЧЕСКИХ ФУНКЦИЙ</t>
   </si>
@@ -482,11 +482,20 @@
   <si>
     <t>y</t>
   </si>
+  <si>
+    <t>g(x) = ln|x|+sin(x)-3e⁻ˣ</t>
+  </si>
+  <si>
+    <t>g(x)</t>
+  </si>
+  <si>
+    <t>f(x)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
@@ -560,7 +569,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -568,11 +577,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -626,6 +650,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -653,7 +678,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -672,7 +703,595 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ru-RU">
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t>График</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="ru-RU" baseline="0">
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t> функции </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0">
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t>f(x)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.32399300087489064"/>
+          <c:y val="3.2407407407407406E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Лист2!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>f(x)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Лист2!$D$3:$D$43</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.85</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.65</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-0.45</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.39999999999999902</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.34999999999999898</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-0.29999999999999899</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-0.249999999999999</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.19999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-0.149999999999999</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-9.9999999999999006E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-4.9999999999998997E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.65</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.85</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Лист2!$E$3:$E$43</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>-0.72425758523368178</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.72010320285080409</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.70287136140288509</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.67514395735442978</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.6394045175293499</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.59777826458536898</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.55193336016125727</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.50308556914647218</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.45205450868967822</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-0.39933621401526054</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.34517222095309169</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-0.28960578030948059</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.2325210910597714</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.17366237598356937</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-0.11262616164788929</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-4.8809458319279783E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.8732186583274989E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>9.1650943184954689E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.17337686377761746</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.27344840369580098</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.27334613570947991</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.17286267218508983</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>9.0748092465927313E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.830516542332826E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-4.6706437684615618E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-0.10458621641912458</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-0.15496429137276563</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-0.19735475219368787</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-0.23144090454032354</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-0.25720936187535648</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>-0.27497967178838256</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>-0.28536332421178168</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>-0.2891836451434826</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>-0.28738373438204734</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>-0.28094191382331674</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>-0.2708053856859734</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>-0.2578453472370949</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>-0.24283185903817561</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>-0.22642431915098701</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>-0.20917280805207569</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="281623520"/>
+        <c:axId val="281623128"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="281623520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="281623128"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="281623128"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="281623520"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="ru-RU"/>
   <c:roundedCorners val="0"/>
@@ -933,7 +1552,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-7BC6-4751-9BD0-5264DEF23488}"/>
             </c:ext>
@@ -947,11 +1566,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="198869376"/>
-        <c:axId val="194172912"/>
+        <c:axId val="237817616"/>
+        <c:axId val="134725248"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="198869376"/>
+        <c:axId val="237817616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1071,12 +1690,12 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="194172912"/>
+        <c:crossAx val="134725248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="194172912"/>
+        <c:axId val="134725248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1196,7 +1815,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="198869376"/>
+        <c:crossAx val="237817616"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1285,7 +1904,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1860,6 +3035,397 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>42862</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1065933" cy="265329"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="TextBox 1"/>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1943100" y="42862"/>
+              <a:ext cx="1065933" cy="265329"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1000">
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>f(x)=</a:t>
+              </a:r>
+              <a14:m>
+                <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:f>
+                    <m:fPr>
+                      <m:ctrlPr>
+                        <a:rPr lang="en-US" sz="1000" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                      </m:ctrlPr>
+                    </m:fPr>
+                    <m:num>
+                      <m:func>
+                        <m:funcPr>
+                          <m:ctrlPr>
+                            <a:rPr lang="en-US" sz="1000" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:funcPr>
+                        <m:fName>
+                          <m:r>
+                            <m:rPr>
+                              <m:sty m:val="p"/>
+                            </m:rPr>
+                            <a:rPr lang="en-US" sz="1000" i="0">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>cos</m:t>
+                          </m:r>
+                        </m:fName>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>2</m:t>
+                          </m:r>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>𝑥</m:t>
+                          </m:r>
+                        </m:e>
+                      </m:func>
+                      <m:r>
+                        <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:rad>
+                        <m:radPr>
+                          <m:degHide m:val="on"/>
+                          <m:ctrlPr>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:radPr>
+                        <m:deg/>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>2</m:t>
+                          </m:r>
+                          <m:d>
+                            <m:dPr>
+                              <m:begChr m:val="|"/>
+                              <m:endChr m:val="|"/>
+                              <m:ctrlPr>
+                                <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                </a:rPr>
+                              </m:ctrlPr>
+                            </m:dPr>
+                            <m:e>
+                              <m:func>
+                                <m:funcPr>
+                                  <m:ctrlPr>
+                                    <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                      <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                    </a:rPr>
+                                  </m:ctrlPr>
+                                </m:funcPr>
+                                <m:fName>
+                                  <m:r>
+                                    <m:rPr>
+                                      <m:sty m:val="p"/>
+                                    </m:rPr>
+                                    <a:rPr lang="en-US" sz="1000" b="0" i="0">
+                                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                      <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                    </a:rPr>
+                                    <m:t>sin</m:t>
+                                  </m:r>
+                                </m:fName>
+                                <m:e>
+                                  <m:r>
+                                    <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                      <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                    </a:rPr>
+                                    <m:t>2</m:t>
+                                  </m:r>
+                                  <m:r>
+                                    <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                      <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                      <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                    </a:rPr>
+                                    <m:t>𝑥</m:t>
+                                  </m:r>
+                                </m:e>
+                              </m:func>
+                            </m:e>
+                          </m:d>
+                        </m:e>
+                      </m:rad>
+                    </m:num>
+                    <m:den>
+                      <m:r>
+                        <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>3</m:t>
+                      </m:r>
+                      <m:sSup>
+                        <m:sSupPr>
+                          <m:ctrlPr>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:sSupPr>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>𝑥</m:t>
+                          </m:r>
+                        </m:e>
+                        <m:sup>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>3</m:t>
+                          </m:r>
+                        </m:sup>
+                      </m:sSup>
+                      <m:r>
+                        <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>+2</m:t>
+                      </m:r>
+                      <m:sSup>
+                        <m:sSupPr>
+                          <m:ctrlPr>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                          </m:ctrlPr>
+                        </m:sSupPr>
+                        <m:e>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>𝑒</m:t>
+                          </m:r>
+                        </m:e>
+                        <m:sup>
+                          <m:r>
+                            <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>−</m:t>
+                          </m:r>
+                          <m:sSup>
+                            <m:sSupPr>
+                              <m:ctrlPr>
+                                <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                </a:rPr>
+                              </m:ctrlPr>
+                            </m:sSupPr>
+                            <m:e>
+                              <m:r>
+                                <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                </a:rPr>
+                                <m:t>𝑥</m:t>
+                              </m:r>
+                            </m:e>
+                            <m:sup>
+                              <m:r>
+                                <a:rPr lang="en-US" sz="1000" b="0" i="1">
+                                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                                </a:rPr>
+                                <m:t>2</m:t>
+                              </m:r>
+                            </m:sup>
+                          </m:sSup>
+                        </m:sup>
+                      </m:sSup>
+                    </m:den>
+                  </m:f>
+                </m:oMath>
+              </a14:m>
+              <a:endParaRPr lang="ru-RU" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="TextBox 1"/>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1943100" y="42862"/>
+              <a:ext cx="1065933" cy="265329"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1000">
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>f(x)=</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1000" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(cos⁡</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1000" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>2𝑥−√(2|sin⁡2𝑥 | ))/(3𝑥^3+2𝑒^(−𝑥^2 ) )</a:t>
+              </a:r>
+              <a:endParaRPr lang="ru-RU" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Диаграмма 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
@@ -2163,14 +3729,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -2260,14 +3826,14 @@
       <c r="AC3" s="1"/>
     </row>
     <row r="4" spans="1:29" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -2429,16 +3995,16 @@
       <c r="AC8" s="1"/>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="23"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="28"/>
+      <c r="F9" s="29"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -2464,10 +4030,10 @@
       <c r="AC9" s="1"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="30"/>
       <c r="C10" s="1"/>
       <c r="D10" s="2"/>
       <c r="E10" s="5">
@@ -2502,11 +4068,11 @@
       <c r="AC10" s="1"/>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="2"/>
       <c r="E11" s="5">
         <f>PI()*(B7^2)</f>
@@ -2540,11 +4106,11 @@
       <c r="AC11" s="1"/>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
       <c r="D12" s="2"/>
       <c r="E12" s="5">
         <f>PI()*B7*E10</f>
@@ -2578,11 +4144,11 @@
       <c r="AC12" s="1"/>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
       <c r="D13" s="2"/>
       <c r="E13" s="5">
         <f>E11+E12</f>
@@ -2616,10 +4182,10 @@
       <c r="AC13" s="1"/>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="23"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="6"/>
       <c r="D14" s="2"/>
       <c r="E14" s="5">
@@ -2654,10 +4220,10 @@
       <c r="AC14" s="1"/>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="23"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="6"/>
       <c r="D15" s="2"/>
       <c r="E15" s="5"/>
@@ -3490,12 +5056,14 @@
   <dimension ref="A1:X44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
+    <row r="1" spans="1:24" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="33"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -3517,11 +5085,19 @@
       <c r="X1" s="2"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
+      <c r="A2" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>68</v>
+      </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="D2" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>69</v>
+      </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -3543,11 +5119,21 @@
       <c r="X2" s="2"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="A3" s="34">
+        <v>-10</v>
+      </c>
+      <c r="B3" s="34">
+        <f>LN(ABS(A3)) + SIN(A3) - 3*EXP(-A3)</f>
+        <v>-66076.550778216275</v>
+      </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="D3" s="34">
+        <v>-1</v>
+      </c>
+      <c r="E3" s="34">
+        <f>(COS(2*D3) - SQRT(2*ABS(SIN(2*D3)))) / (3*D3^3 + 2*EXP(-D3^2))</f>
+        <v>-0.72425758523368178</v>
+      </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -3569,11 +5155,21 @@
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
+      <c r="A4" s="34">
+        <v>-9</v>
+      </c>
+      <c r="B4" s="34">
+        <f>LN(ABS(A4)) + SIN(A4) - 3*EXP(-A4)</f>
+        <v>-24307.46667663406</v>
+      </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="D4" s="34">
+        <v>-0.95</v>
+      </c>
+      <c r="E4" s="34">
+        <f t="shared" ref="E4:E43" si="0">(COS(2*D4) - SQRT(2*ABS(SIN(2*D4)))) / (3*D4^3 + 2*EXP(-D4^2))</f>
+        <v>-0.72010320285080409</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -3595,11 +5191,21 @@
       <c r="X4" s="2"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="A5" s="34">
+        <v>-8</v>
+      </c>
+      <c r="B5" s="34">
+        <f>LN(ABS(A5)) + SIN(A5) - 3*EXP(-A5)</f>
+        <v>-8941.7838778301284</v>
+      </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="D5" s="34">
+        <v>-0.9</v>
+      </c>
+      <c r="E5" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.70287136140288509</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -3621,11 +5227,21 @@
       <c r="X5" s="2"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
+      <c r="A6" s="34">
+        <v>-7</v>
+      </c>
+      <c r="B6" s="34">
+        <f>LN(ABS(A6)) + SIN(A6) - 3*EXP(-A6)</f>
+        <v>-3288.6105517350388</v>
+      </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="D6" s="34">
+        <v>-0.85</v>
+      </c>
+      <c r="E6" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.67514395735442978</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -3647,11 +5263,21 @@
       <c r="X6" s="2"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="34">
+        <v>-6</v>
+      </c>
+      <c r="B7" s="34">
+        <f>LN(ABS(A7)) + SIN(A7) - 3*EXP(-A7)</f>
+        <v>-1208.2152055107783</v>
+      </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="D7" s="34">
+        <v>-0.8</v>
+      </c>
+      <c r="E7" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.6394045175293499</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -3673,11 +5299,21 @@
       <c r="X7" s="2"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="34">
+        <v>-5</v>
+      </c>
+      <c r="B8" s="34">
+        <f>LN(ABS(A8)) + SIN(A8) - 3*EXP(-A8)</f>
+        <v>-442.67111512063252</v>
+      </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="D8" s="34">
+        <v>-0.75</v>
+      </c>
+      <c r="E8" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.59777826458536898</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -3699,11 +5335,21 @@
       <c r="X8" s="2"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+      <c r="A9" s="34">
+        <v>-4</v>
+      </c>
+      <c r="B9" s="34">
+        <f>LN(ABS(A9)) + SIN(A9) - 3*EXP(-A9)</f>
+        <v>-161.65135324300488</v>
+      </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="D9" s="34">
+        <v>-0.7</v>
+      </c>
+      <c r="E9" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.55193336016125727</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -3725,11 +5371,21 @@
       <c r="X9" s="2"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
+      <c r="A10" s="34">
+        <v>-3</v>
+      </c>
+      <c r="B10" s="34">
+        <f>LN(ABS(A10)) + SIN(A10) - 3*EXP(-A10)</f>
+        <v>-59.299118488954761</v>
+      </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="D10" s="34">
+        <v>-0.65</v>
+      </c>
+      <c r="E10" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.50308556914647218</v>
+      </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -3751,11 +5407,21 @@
       <c r="X10" s="2"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+      <c r="A11" s="34">
+        <v>-2</v>
+      </c>
+      <c r="B11" s="34">
+        <f>LN(ABS(A11)) + SIN(A11) - 3*EXP(-A11)</f>
+        <v>-22.383318543057687</v>
+      </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="D11" s="34">
+        <v>-0.6</v>
+      </c>
+      <c r="E11" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.45205450868967822</v>
+      </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -3777,11 +5443,21 @@
       <c r="X11" s="2"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="34">
+        <v>-1</v>
+      </c>
+      <c r="B12" s="34">
+        <f>LN(ABS(A12)) + SIN(A12) - 3*EXP(-A12)</f>
+        <v>-8.9963164701850324</v>
+      </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="D12" s="34">
+        <v>-0.55000000000000004</v>
+      </c>
+      <c r="E12" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.39933621401526054</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -3803,11 +5479,21 @@
       <c r="X12" s="2"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="34">
+        <v>1</v>
+      </c>
+      <c r="B13" s="34">
+        <f>LN(ABS(A13)) + SIN(A13) - 3*EXP(-A13)</f>
+        <v>-0.2621673387064305</v>
+      </c>
       <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="D13" s="34">
+        <v>-0.5</v>
+      </c>
+      <c r="E13" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.34517222095309169</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -3829,11 +5515,21 @@
       <c r="X13" s="2"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="34">
+        <v>2</v>
+      </c>
+      <c r="B14" s="34">
+        <f>LN(ABS(A14)) + SIN(A14) - 3*EXP(-A14)</f>
+        <v>1.1964387576757889</v>
+      </c>
       <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="D14" s="34">
+        <v>-0.45</v>
+      </c>
+      <c r="E14" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.28960578030948059</v>
+      </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -3855,11 +5551,21 @@
       <c r="X14" s="2"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="34">
+        <v>3</v>
+      </c>
+      <c r="B15" s="34">
+        <f>LN(ABS(A15)) + SIN(A15) - 3*EXP(-A15)</f>
+        <v>1.0903710916243852</v>
+      </c>
       <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="D15" s="34">
+        <v>-0.39999999999999902</v>
+      </c>
+      <c r="E15" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.2325210910597714</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -3881,11 +5587,21 @@
       <c r="X15" s="2"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="34">
+        <v>4</v>
+      </c>
+      <c r="B16" s="34">
+        <f>LN(ABS(A16)) + SIN(A16) - 3*EXP(-A16)</f>
+        <v>0.57454494914575982</v>
+      </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="D16" s="34">
+        <v>-0.34999999999999898</v>
+      </c>
+      <c r="E16" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.17366237598356937</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -3907,11 +5623,21 @@
       <c r="X16" s="2"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="34">
+        <v>5</v>
+      </c>
+      <c r="B17" s="34">
+        <f>LN(ABS(A17)) + SIN(A17) - 3*EXP(-A17)</f>
+        <v>0.6302997967737054</v>
+      </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="D17" s="34">
+        <v>-0.29999999999999899</v>
+      </c>
+      <c r="E17" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.11262616164788929</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -3933,11 +5659,21 @@
       <c r="X17" s="2"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="34">
+        <v>6</v>
+      </c>
+      <c r="B18" s="34">
+        <f>LN(ABS(A18)) + SIN(A18) - 3*EXP(-A18)</f>
+        <v>1.5049077144991301</v>
+      </c>
       <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="D18" s="34">
+        <v>-0.249999999999999</v>
+      </c>
+      <c r="E18" s="34">
+        <f t="shared" si="0"/>
+        <v>-4.8809458319279783E-2</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -3959,11 +5695,21 @@
       <c r="X18" s="2"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="A19" s="34">
+        <v>7</v>
+      </c>
+      <c r="B19" s="34">
+        <f>LN(ABS(A19)) + SIN(A19) - 3*EXP(-A19)</f>
+        <v>2.6001611018774389</v>
+      </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="D19" s="34">
+        <v>-0.19999999999999901</v>
+      </c>
+      <c r="E19" s="34">
+        <f t="shared" si="0"/>
+        <v>1.8732186583274989E-2</v>
+      </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -3985,11 +5731,21 @@
       <c r="X19" s="2"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="A20" s="34">
+        <v>8</v>
+      </c>
+      <c r="B20" s="34">
+        <f>LN(ABS(A20)) + SIN(A20) - 3*EXP(-A20)</f>
+        <v>3.06779340041951</v>
+      </c>
       <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="D20" s="34">
+        <v>-0.149999999999999</v>
+      </c>
+      <c r="E20" s="34">
+        <f t="shared" si="0"/>
+        <v>9.1650943184954689E-2</v>
+      </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -4011,11 +5767,21 @@
       <c r="X20" s="2"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="A21" s="34">
+        <v>9</v>
+      </c>
+      <c r="B21" s="34">
+        <f>LN(ABS(A21)) + SIN(A21) - 3*EXP(-A21)</f>
+        <v>2.608972833165716</v>
+      </c>
       <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="D21" s="34">
+        <v>-9.9999999999999006E-2</v>
+      </c>
+      <c r="E21" s="34">
+        <f t="shared" si="0"/>
+        <v>0.17337686377761746</v>
+      </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -4037,11 +5803,21 @@
       <c r="X21" s="2"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
+      <c r="A22" s="34">
+        <v>10</v>
+      </c>
+      <c r="B22" s="34">
+        <f>LN(ABS(A22)) + SIN(A22) - 3*EXP(-A22)</f>
+        <v>1.7584277823153887</v>
+      </c>
       <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+      <c r="D22" s="34">
+        <v>-4.9999999999998997E-2</v>
+      </c>
+      <c r="E22" s="34">
+        <f t="shared" si="0"/>
+        <v>0.27344840369580098</v>
+      </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -4063,11 +5839,14 @@
       <c r="X22" s="2"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
+      <c r="D23" s="34">
+        <v>0</v>
+      </c>
+      <c r="E23" s="34">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -4092,8 +5871,13 @@
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="D24" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="E24" s="34">
+        <f t="shared" si="0"/>
+        <v>0.27334613570947991</v>
+      </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -4118,8 +5902,13 @@
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
+      <c r="D25" s="34">
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="34">
+        <f t="shared" si="0"/>
+        <v>0.17286267218508983</v>
+      </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -4144,8 +5933,13 @@
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
+      <c r="D26" s="34">
+        <v>0.15</v>
+      </c>
+      <c r="E26" s="34">
+        <f t="shared" si="0"/>
+        <v>9.0748092465927313E-2</v>
+      </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -4170,8 +5964,13 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="D27" s="34">
+        <v>0.2</v>
+      </c>
+      <c r="E27" s="34">
+        <f t="shared" si="0"/>
+        <v>1.830516542332826E-2</v>
+      </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -4196,8 +5995,13 @@
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="D28" s="34">
+        <v>0.25</v>
+      </c>
+      <c r="E28" s="34">
+        <f t="shared" si="0"/>
+        <v>-4.6706437684615618E-2</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -4222,8 +6026,13 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="D29" s="34">
+        <v>0.3</v>
+      </c>
+      <c r="E29" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.10458621641912458</v>
+      </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -4248,8 +6057,13 @@
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="D30" s="34">
+        <v>0.35</v>
+      </c>
+      <c r="E30" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.15496429137276563</v>
+      </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -4274,8 +6088,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
+      <c r="D31" s="34">
+        <v>0.4</v>
+      </c>
+      <c r="E31" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.19735475219368787</v>
+      </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -4300,8 +6119,13 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
+      <c r="D32" s="34">
+        <v>0.45</v>
+      </c>
+      <c r="E32" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.23144090454032354</v>
+      </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -4326,8 +6150,13 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="D33" s="34">
+        <v>0.5</v>
+      </c>
+      <c r="E33" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.25720936187535648</v>
+      </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -4352,8 +6181,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
+      <c r="D34" s="34">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E34" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.27497967178838256</v>
+      </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
@@ -4378,8 +6212,13 @@
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
+      <c r="D35" s="34">
+        <v>0.6</v>
+      </c>
+      <c r="E35" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.28536332421178168</v>
+      </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
@@ -4404,8 +6243,13 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="D36" s="34">
+        <v>0.65</v>
+      </c>
+      <c r="E36" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.2891836451434826</v>
+      </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -4430,8 +6274,13 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+      <c r="D37" s="34">
+        <v>0.7</v>
+      </c>
+      <c r="E37" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.28738373438204734</v>
+      </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -4456,8 +6305,13 @@
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="D38" s="34">
+        <v>0.75</v>
+      </c>
+      <c r="E38" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.28094191382331674</v>
+      </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -4482,8 +6336,13 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="D39" s="34">
+        <v>0.8</v>
+      </c>
+      <c r="E39" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.2708053856859734</v>
+      </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -4508,8 +6367,13 @@
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="D40" s="34">
+        <v>0.85</v>
+      </c>
+      <c r="E40" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.2578453472370949</v>
+      </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
@@ -4534,8 +6398,13 @@
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
+      <c r="D41" s="34">
+        <v>0.9</v>
+      </c>
+      <c r="E41" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.24283185903817561</v>
+      </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
@@ -4560,8 +6429,13 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="D42" s="34">
+        <v>0.95</v>
+      </c>
+      <c r="E42" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.22642431915098701</v>
+      </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -4586,8 +6460,13 @@
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
+      <c r="D43" s="34">
+        <v>1</v>
+      </c>
+      <c r="E43" s="34">
+        <f t="shared" si="0"/>
+        <v>-0.20917280805207569</v>
+      </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
@@ -4635,7 +6514,12 @@
       <c r="X44" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4654,7 +6538,7 @@
       </c>
       <c r="B1" s="11">
         <f ca="1">TODAY()</f>
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -4663,7 +6547,7 @@
       </c>
       <c r="B2" s="12">
         <f ca="1">YEARFRAC(B1,A1)</f>
-        <v>18.138888888888889</v>
+        <v>18.141666666666666</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -4883,9 +6767,9 @@
       <c r="U6" s="1"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" s="31"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -6906,10 +8790,10 @@
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="23" t="s">
         <v>66</v>
       </c>
       <c r="C4" s="2"/>

</xml_diff>